<commit_message>
Phase 1.16 — Binary uploads + Flow/Audit UX (19 sub-tasks)
Core feature (10):
- Backend `uploads` table + on-disk store in data/uploads/<uuid>
- POST/GET/DELETE routes (express.raw, 10MB cap, x-filename header)
- timing.ts binary body builder: raw bytes or multipart/form-data
- Shared BinaryBodyEditor wired into URL / Flow / Prereq editors
- Flow "Run Now" auto-runs prereq chain first (force=true)
- Audit defaults to current-state snapshot (no re-checks)

UX overhaul (9):
- BinaryBodyEditor redesigned as full dropzone with drag-drop
- Real upload progress bar (XHR onprogress %)
- Client-side 10MB size guard
- Selected-file card with thumb, ext badge, inline actions
- Raw vs Form-field radio toggle replaces cryptic empty-fieldname
- Auto-dismissing success/error banners
- Collapsible project upload library
- FlowCard prereq-running banner ("Refreshing access tokens…")
- Audit button copy: "Snapshot & report" + clearer tooltip

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-tracker.xlsx
+++ b/project-tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$1:$J$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$1:$J$155</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J136"/>
+  <dimension ref="A1:J155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4858,8 +4858,616 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>16.1</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>Backend: uploads table + on-disk storage in data/uploads/&lt;uuid&gt;</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>One row per file; bytes live on disk not in SQLite</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>16.2</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>Backend: paths.ts helper centralises UPLOADS_DIR + per-id path</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>Shared by index.ts upload routes and timing.ts body builder</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>16.3</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>Backend: POST/GET/DELETE routes (express.raw 10MB cap; URL-encoded x-filename header)</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>No multer dependency; raw bytes go straight to disk</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>16.4</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>Backend: store CRUD (createUpload/getUpload/listUploadsByProject/deleteUpload)</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>Mirrors existing row-mapper pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>16.5</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>Backend: bodyType=binary in timing.ts parses {uploadId fieldName?} body and builds raw or multipart</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>Empty fieldName = raw bytes; set = multipart/form-data</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>16.6</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Frontend: shared BinaryBodyEditor with file picker / image preview / field-name / existing-uploads picker</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>Single component reused by URL + Flow step + Prereq step editors</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>16.7</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>Frontend: Binary tab added to all three body editors (URL form / Flow step / Prereq step)</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>Discoverable in same Body tab as JSON / Raw / form-data</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>16.8</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>UX: Run Now on a Flow auto-runs the prereq chain first with force=true</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>Avoids spurious failures from stale auth tokens</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>16.9</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>UX: Audit renamed Generate report - snapshots current state; ?refresh=true opt-in for re-check</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>Used to re-run everything; now defaults to fast snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>16.10</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Smoke test: upload list readback delete round-trip via curl</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>Verified POST returns id; GET streams bytes; DELETE 204s</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>16.11</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>Frontend: BinaryBodyEditor redesigned as full dropzone (click or drag-drop) with hover/dragover states</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>Old "Upload file" button was ambiguous - users were unsure whether click would open picker or upload</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>16.12</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>Frontend: real upload progress bar (XHR onprogress with %) replaces opaque "Uploading..." text</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>Live feedback for large files; no more guessing if it hung</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>16.13</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>Frontend: client-side max-size guard (10MB) shows inline error before hitting server</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>Saves a wasted upload + slow round-trip for over-cap files</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>16.14</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Frontend: selected file card with thumb / ext badge / size / inline replace+delete actions</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>Replaces compact row that buried the actions</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>16.15</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>Frontend: explicit Raw vs Form-field radio toggle (vs cryptic empty-fieldname meaning)</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>Beginners no longer have to read help text to understand what empty fieldname does</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>16.16</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Frontend: success+error banners with auto-dismiss (3s) after upload completes or fails</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>Confirms upload succeeded without forcing scroll to bottom</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>16.17</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>Frontend: project upload library collapsed by default (toggle to expand)</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>Cleaner default view when project has many uploads</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>16.18</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>Frontend: Flow card surfaces "Refreshing access tokens..." banner during prereq phase</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>Previously only a PREREQ pill switch - banner makes the wait self-explanatory</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>16.19</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>Frontend: Audit button copy "Snapshot &amp; report" + tooltip clarifies no re-checks happen</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>Button now reads as the action it performs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J136"/>
+  <autoFilter ref="A1:J155"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rebuild BinaryBodyEditor in Postman style
Per user feedback: dropzone + radio toggle + banners felt out of
place vs the rest of the Postman-style editor surfaces.

- Replace dropzone with compact "Select File" button + inline
  filename + clear (x) — matches Postman's binary body tab layout
- Replace radio toggle with a plain "Field name (optional)" input
  (empty = raw bytes, set = multipart) — same single-tab semantic
  Postman uses
- Replace big success/error banners with subdued inline left-bar
  error text
- Library list is now tight rows (thumb / name / size / check
  for active / hover-only delete) instead of bordered card grid
- Upload progress is a thin 3px bar under the file row, not a
  bordered progress card
</commit_message>
<xml_diff>
--- a/project-tracker.xlsx
+++ b/project-tracker.xlsx
@@ -5191,7 +5191,7 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>Frontend: BinaryBodyEditor redesigned as full dropzone (click or drag-drop) with hover/dragover states</t>
+          <t>Frontend: BinaryBodyEditor rebuilt in Postman style - Select File button + inline filename + clear x; compact utilitarian row</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>Old "Upload file" button was ambiguous - users were unsure whether click would open picker or upload</t>
+          <t>User feedback: oversized dropzone felt out of place vs rest of Postman-like editor</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Frontend: selected file card with thumb / ext badge / size / inline replace+delete actions</t>
+          <t>Frontend: inline filename + size display with x clear button (Postman binary tab layout)</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>Replaces compact row that buried the actions</t>
+          <t>Matches Postman binary body editor exactly</t>
         </is>
       </c>
     </row>
@@ -5319,7 +5319,7 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>Frontend: explicit Raw vs Form-field radio toggle (vs cryptic empty-fieldname meaning)</t>
+          <t>Frontend: Field name (optional) inline input - empty = raw bytes / set = multipart</t>
         </is>
       </c>
       <c r="D151" s="3" t="inlineStr">
@@ -5334,7 +5334,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>Beginners no longer have to read help text to understand what empty fieldname does</t>
+          <t>Postman-style single-tab semantic instead of radio toggle</t>
         </is>
       </c>
     </row>
@@ -5351,7 +5351,7 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>Frontend: success+error banners with auto-dismiss (3s) after upload completes or fails</t>
+          <t>Frontend: inline left-bar error message (no large banners)</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
@@ -5366,7 +5366,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>Confirms upload succeeded without forcing scroll to bottom</t>
+          <t>Postman-style subdued inline feedback</t>
         </is>
       </c>
     </row>
@@ -5383,7 +5383,7 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>Frontend: project upload library collapsed by default (toggle to expand)</t>
+          <t>Frontend: project uploads library - collapsible tight rows with thumb/ext / check for active / hover-only delete</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
@@ -5398,7 +5398,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>Cleaner default view when project has many uploads</t>
+          <t>Postman-style tight row list</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix × on selected file to delete from project (not just unbind)
User report: clicking × on the selected file row only cleared
the step's reference — the file still appeared in "Project uploads"
which was confusing.

× now calls DELETE /api/uploads/:id (with confirm), removes the
file from both the project library and the current selection.
The library trash icon already did this; now both paths share
the same delete handler.
</commit_message>
<xml_diff>
--- a/project-tracker.xlsx
+++ b/project-tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$1:$J$155</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$1:$J$156</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J155"/>
+  <dimension ref="A1:J156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5466,8 +5466,40 @@
         </is>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>16.20</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Fix: x button on selected file now deletes from project (not just unbinds from step)</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>User reported: deleted file still appeared in Project uploads list</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J155"/>
+  <autoFilter ref="A1:J156"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
In-UI two-click confirm for upload delete
Replace native window.confirm() with the same two-click inline
pattern used elsewhere in the app (Phase 1.15.4 for step delete).

- × on selected file morphs into red pulsing "Click to confirm"
- 🗑 on library rows morphs into red pulsing "Confirm?"
- Either one auto-resets after 4 seconds without a second click
- Single confirmingId state — arming a different row resets the
  previous one automatically

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-tracker.xlsx
+++ b/project-tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$1:$J$156</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$1:$J$157</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J156"/>
+  <dimension ref="A1:J157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5498,8 +5498,40 @@
         </is>
       </c>
     </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>16.21</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>Replace native window.confirm for upload delete with two-click inline confirm (matches existing step-delete pattern from 15.4)</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>Stays in-app instead of jumping to browser modal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J156"/>
+  <autoFilter ref="A1:J157"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Show live prereq progress during flow Run Now
The "🔑 Refreshing access tokens…" banner was opaque — users
couldn't tell if the prereq was progressing or hung. Same poll
loop already had the data; we just weren't surfacing it.

- New prereqProgress state {completed, total, live}
- Updated inside the existing poll loop from pr.stepResults.length
  and pr.liveStep (no extra requests)
- Banner now renders: filling background bar, "step N of M",
  N/M done · X% counter, and retry chip when an attempt is
  retrying or backing off
- Matches the existing flow-progress visual language so the
  prereq phase doesn't look like a different system

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-tracker.xlsx
+++ b/project-tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$1:$J$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$1:$J$158</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J157"/>
+  <dimension ref="A1:J158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5530,8 +5530,40 @@
         </is>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>16.22</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>Prereq banner now shows live step-N-of-M + completed count + retry chip + filling progress bar</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>Previously opaque - users couldn't tell if prereq was progressing or stuck</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J157"/>
+  <autoFilter ref="A1:J158"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Show full prereq progress UI when Flow Run-now triggers chain
FlowCard's "Run now" now lifts the prereq runId up to ProjectView,
which passes it to PrereqsPanel as externalRunId. The panel re-uses
its existing handleRun loop (with the lifted id instead of starting
a fresh chain), auto-expands, and renders the same complete progress
bar + step-by-step rows that appear when the user clicks the panel's
own Run-now. FlowCard keeps its inline banner for in-context feedback.
</commit_message>
<xml_diff>
--- a/project-tracker.xlsx
+++ b/project-tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$1:$J$158</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$1:$J$159</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J158"/>
+  <dimension ref="A1:J159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5562,8 +5562,40 @@
         </is>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>16.23</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.16 - Binary uploads + UX tightening</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>FlowCard Run-now lifts prereq runId up so PrereqsPanel attaches and shows the full step-by-step progress UI (matching panel's own Run-now behaviour)</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr">
+        <is>
+          <t>User feedback: panel's complete bar only appeared when prereq triggered from the panel itself</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J158"/>
+  <autoFilter ref="A1:J159"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phase 1.24 — Export project to OpenAPI / Swagger spec (YAML + JSON)
Hybrid encoding: every HTTP step (URL monitor, flow step, prereq) becomes
a Swagger paths entry carrying our orchestration metadata in x-mon-*
extensions, AND a top-level x-mon-flows side-band preserves every flow
(including Compute and Loop steps) in position order so the export is
fully round-trippable. New GET /api/projects/:id/export/openapi?format=yaml|json
endpoint streams the spec as an attachment. New "📥 Export to Swagger"
button in ProjectView triggers the download. Spec is deterministic
(alphabetical paths, position-ordered flow steps) so re-exports diff cleanly.
</commit_message>
<xml_diff>
--- a/project-tracker.xlsx
+++ b/project-tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$1:$J$301</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tracker'!$A$1:$J$308</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J301"/>
+  <dimension ref="A1:J308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10138,8 +10138,232 @@
         </is>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" s="2" t="inlineStr">
+        <is>
+          <t>24.1</t>
+        </is>
+      </c>
+      <c r="B302" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.24 - Export to Swagger/OpenAPI</t>
+        </is>
+      </c>
+      <c r="C302" s="2" t="inlineStr">
+        <is>
+          <t>Backend openapiExport.ts (new): pure transform buildOpenAPISpec(project, urls, flows, prereqs); helpers - splitServerAndPath (URL() with {{var}} placeholder protection) + toOpenAPIPathKey ({{a.b}}-&gt;{a_b} so dotted vars stay distinct) + templateVarsToPathParams + extractServers (filters compute://step + loop://step sentinels) + buildSecuritySchemes (Authorization+Bearer -&gt; type:http scheme:bearer; else type:apiKey in:header name:headerName) + buildOperationForUrl/FlowStep/Prereq + mergeOperation (collision-safe path+method append with #id-slice alias key) + buildXMonFlow (full side-band with stepType+level+forEach+compute) + sortKeys (deterministic alphabetical paths); zero DB access</t>
+        </is>
+      </c>
+      <c r="D302" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E302" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F302" s="2" t="inlineStr">
+        <is>
+          <t>Pure transform - no side effects testable in isolation</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="2" t="inlineStr">
+        <is>
+          <t>24.2</t>
+        </is>
+      </c>
+      <c r="B303" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.24 - Export to Swagger/OpenAPI</t>
+        </is>
+      </c>
+      <c r="C303" s="2" t="inlineStr">
+        <is>
+          <t>Backend index.ts: new GET /api/projects/:id/export/openapi?format=yaml|json (defaults YAML); reuses getProject + listUrlsByProject + listFlowsByProject + getFlowWithSteps + listPrereqSteps; emits via js-yaml dump (lineWidth 120 noRefs true sortKeys false) or JSON.stringify(spec,null,2); content-disposition attachment filename=&lt;slug&gt;-openapi.&lt;ext&gt; triggers browser download</t>
+        </is>
+      </c>
+      <c r="D303" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E303" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F303" s="2" t="inlineStr">
+        <is>
+          <t>Mirrors existing report-download endpoint pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="2" t="inlineStr">
+        <is>
+          <t>24.3</t>
+        </is>
+      </c>
+      <c r="B304" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.24 - Export to Swagger/OpenAPI</t>
+        </is>
+      </c>
+      <c r="C304" s="2" t="inlineStr">
+        <is>
+          <t>Backend package.json: added js-yaml@^4.1.0 + @types/js-yaml@^4.0.9; same lib will handle import parsing later picked once for round-trip symmetry</t>
+        </is>
+      </c>
+      <c r="D304" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E304" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F304" s="2" t="inlineStr">
+        <is>
+          <t>One dep covers both directions</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="2" t="inlineStr">
+        <is>
+          <t>24.4</t>
+        </is>
+      </c>
+      <c r="B305" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.24 - Export to Swagger/OpenAPI</t>
+        </is>
+      </c>
+      <c r="C305" s="2" t="inlineStr">
+        <is>
+          <t>Frontend api.ts: new exportProjectOpenAPI(projectId,format) returning {blob,filename}; parses content-disposition for server-suggested filename falls back to openapi.&lt;ext&gt;</t>
+        </is>
+      </c>
+      <c r="D305" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E305" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F305" s="2" t="inlineStr">
+        <is>
+          <t>Same fetch pattern as audit-report download</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="2" t="inlineStr">
+        <is>
+          <t>24.5</t>
+        </is>
+      </c>
+      <c r="B306" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.24 - Export to Swagger/OpenAPI</t>
+        </is>
+      </c>
+      <c r="C306" s="2" t="inlineStr">
+        <is>
+          <t>Frontend ProjectView.tsx: new 📥 Export to Swagger button in hero-actions between Snapshot and settings icons; handler creates Blob URL triggers temp anchor download revokes URL pushes success/error toast; loading state Spinner + Exporting...; disabled when zero URLs AND zero flows with explanatory tooltip</t>
+        </is>
+      </c>
+      <c r="D306" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E306" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F306" s="2" t="inlineStr">
+        <is>
+          <t>Standard browser download UX no new dep</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="2" t="inlineStr">
+        <is>
+          <t>24.6</t>
+        </is>
+      </c>
+      <c r="B307" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.24 - Export to Swagger/OpenAPI</t>
+        </is>
+      </c>
+      <c r="C307" s="2" t="inlineStr">
+        <is>
+          <t>End-to-end smoke on live CMS/Logitech project: YAML export clean OpenAPI 3.0.3 - servers exactly the 2 real hosts (compute/loop sentinels filtered) + paths alphabetically sorted + /api/getCampaigns and 2 dotted-path-distinct /campaign/{campaign_documentId}/{campaign_locale}/{geo}/... paths + securitySchemes.campaign-api-key={type:http scheme:bearer} correctly derived from Bearer ApiKey + x-mon-flows round-trips Compute mapAddField-&gt;concatArrays(countries,regions) + Loop forEach{campaigns as campaign} + sibling L2 children with forEach{campaign.geos as geo} and full assertions+extractions+level+position; JSON variant parses cleanly; determinism verified (two consecutive exports byte-identical); Default project (no flows 12 hosts) also renders OK</t>
+        </is>
+      </c>
+      <c r="D307" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E307" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F307" s="2" t="inlineStr">
+        <is>
+          <t>Full data-model round-trip via standard format</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>24.7</t>
+        </is>
+      </c>
+      <c r="B308" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.24 - Export to Swagger/OpenAPI</t>
+        </is>
+      </c>
+      <c r="C308" s="2" t="inlineStr">
+        <is>
+          <t>Build clean: backend tsc -b zero output; frontend tsc -b zero output</t>
+        </is>
+      </c>
+      <c r="D308" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E308" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="F308" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid encoding preserves all our orchestration metadata in x-mon-* extensions</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J301"/>
+  <autoFilter ref="A1:J308"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>